<commit_message>
Fix ROM counter overflow
Fix ROM counter overflow
</commit_message>
<xml_diff>
--- a/MagicWildCardRom_Explaination.xlsx
+++ b/MagicWildCardRom_Explaination.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="164011"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Menu_Rom" sheetId="1" r:id="rId1"/>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="18">
   <si>
     <t>MENU ROM HACKING:</t>
   </si>
@@ -306,6 +306,9 @@
       </rPr>
       <t>0x01)</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
   </si>
 </sst>
 </file>
@@ -2104,7 +2107,7 @@
           <a:pPr algn="l"/>
           <a:r>
             <a:rPr lang="en-US" sz="1100"/>
-            <a:t>- Last 2 Bytes: Dont know (checksum??????)</a:t>
+            <a:t>- Last 2 Bytes: Dont know (checksum???????)</a:t>
           </a:r>
         </a:p>
       </xdr:txBody>
@@ -2475,7 +2478,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:G175"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="16384" width="9.140625" style="2"/>
@@ -2569,6 +2572,11 @@
         <v>11</v>
       </c>
     </row>
+    <row r="175" spans="7:7" x14ac:dyDescent="0.25">
+      <c r="G175" s="2" t="s">
+        <v>17</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>